<commit_message>
chore: update generated risk reports
</commit_message>
<xml_diff>
--- a/reports/risk_summary_report.xlsx
+++ b/reports/risk_summary_report.xlsx
@@ -437,7 +437,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>44747998.01445286</v>
+        <v>44679024.23005211</v>
       </c>
     </row>
     <row r="3">
@@ -447,7 +447,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>44990134.15638334</v>
+        <v>45042229.10782842</v>
       </c>
     </row>
     <row r="4">
@@ -457,7 +457,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2.659121034455398</v>
+        <v>2.663226084735405</v>
       </c>
     </row>
     <row r="5">
@@ -467,7 +467,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>265.9121034455398</v>
+        <v>266.3226084735405</v>
       </c>
     </row>
     <row r="6">
@@ -477,7 +477,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.9981315649627445</v>
+        <v>0.9975266555860837</v>
       </c>
     </row>
     <row r="7">
@@ -487,7 +487,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.0138654625043273</v>
+        <v>0.01440664567053318</v>
       </c>
     </row>
   </sheetData>
@@ -552,10 +552,10 @@
         <v>5.47505244242807</v>
       </c>
       <c r="E2" t="n">
-        <v>4.43555534660091</v>
+        <v>4.477662694227526</v>
       </c>
       <c r="F2" t="n">
-        <v>5.25419398199517</v>
+        <v>5.311641590719916</v>
       </c>
     </row>
     <row r="3">
@@ -574,10 +574,10 @@
         <v>3.877120891187244</v>
       </c>
       <c r="E3" t="n">
-        <v>4.199754875636979</v>
+        <v>4.253189165462305</v>
       </c>
       <c r="F3" t="n">
-        <v>5.420360621597447</v>
+        <v>5.342159931766103</v>
       </c>
     </row>
     <row r="4">
@@ -596,10 +596,10 @@
         <v>6.091241143731888</v>
       </c>
       <c r="E4" t="n">
-        <v>4.455971949434422</v>
+        <v>4.358058760348153</v>
       </c>
       <c r="F4" t="n">
-        <v>5.325800624385948</v>
+        <v>5.300737899927681</v>
       </c>
     </row>
     <row r="5">
@@ -618,10 +618,10 @@
         <v>3.474342866036952</v>
       </c>
       <c r="E5" t="n">
-        <v>4.277905501526317</v>
+        <v>4.336013966921665</v>
       </c>
       <c r="F5" t="n">
-        <v>5.361708803256647</v>
+        <v>5.271519931771315</v>
       </c>
     </row>
     <row r="6">
@@ -640,10 +640,10 @@
         <v>4.494660689508277</v>
       </c>
       <c r="E6" t="n">
-        <v>4.311434716130881</v>
+        <v>4.335267424699744</v>
       </c>
       <c r="F6" t="n">
-        <v>5.313436063917797</v>
+        <v>5.353124444427294</v>
       </c>
     </row>
     <row r="7">
@@ -662,10 +662,10 @@
         <v>2.419253194704907</v>
       </c>
       <c r="E7" t="n">
-        <v>4.390649891506191</v>
+        <v>4.420226544491245</v>
       </c>
       <c r="F7" t="n">
-        <v>5.321019006252739</v>
+        <v>5.341375897130723</v>
       </c>
     </row>
     <row r="8">
@@ -684,10 +684,10 @@
         <v>3.824239977161246</v>
       </c>
       <c r="E8" t="n">
-        <v>4.231793813758297</v>
+        <v>4.205157337143491</v>
       </c>
       <c r="F8" t="n">
-        <v>5.004283853161341</v>
+        <v>5.676544560309382</v>
       </c>
     </row>
   </sheetData>
@@ -723,7 +723,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.6185358762741089</v>
+        <v>0.6175910234451294</v>
       </c>
     </row>
     <row r="3">
@@ -733,7 +733,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.3104948103427887</v>
+        <v>0.3032228350639343</v>
       </c>
     </row>
     <row r="4">
@@ -743,7 +743,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.03987201303243637</v>
+        <v>0.04758356139063835</v>
       </c>
     </row>
     <row r="5">
@@ -753,7 +753,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.009040437638759613</v>
+        <v>0.008828707039356232</v>
       </c>
     </row>
     <row r="6">
@@ -763,7 +763,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.008423496037721634</v>
+        <v>0.008460237644612789</v>
       </c>
     </row>
     <row r="7">
@@ -773,7 +773,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.00815955176949501</v>
+        <v>0.007544185500591993</v>
       </c>
     </row>
     <row r="8">
@@ -783,7 +783,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.005473894067108631</v>
+        <v>0.006769496016204357</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
AI chat bug resolved
</commit_message>
<xml_diff>
--- a/reports/risk_summary_report.xlsx
+++ b/reports/risk_summary_report.xlsx
@@ -437,7 +437,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>44626193.79379303</v>
+        <v>44690948.54481202</v>
       </c>
     </row>
     <row r="3">
@@ -447,7 +447,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>44831206.41361938</v>
+        <v>45104952.27453943</v>
       </c>
     </row>
     <row r="4">
@@ -457,7 +457,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2.666378928031055</v>
+        <v>2.662515490148688</v>
       </c>
     </row>
     <row r="5">
@@ -467,7 +467,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>266.6378928031055</v>
+        <v>266.2515490148688</v>
       </c>
     </row>
     <row r="6">
@@ -477,7 +477,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.9979534841649423</v>
+        <v>0.9982926856845652</v>
       </c>
     </row>
     <row r="7">
@@ -487,7 +487,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.01348675787448883</v>
+        <v>0.01391142606735229</v>
       </c>
     </row>
   </sheetData>
@@ -552,10 +552,10 @@
         <v>5.47505244242807</v>
       </c>
       <c r="E2" t="n">
-        <v>4.361926462023122</v>
+        <v>4.460435789892159</v>
       </c>
       <c r="F2" t="n">
-        <v>5.203403990036204</v>
+        <v>5.24406922412883</v>
       </c>
     </row>
     <row r="3">
@@ -574,10 +574,10 @@
         <v>3.877120891187244</v>
       </c>
       <c r="E3" t="n">
-        <v>4.203636270842431</v>
+        <v>4.196620746756418</v>
       </c>
       <c r="F3" t="n">
-        <v>5.364867078345162</v>
+        <v>5.394565056106587</v>
       </c>
     </row>
     <row r="4">
@@ -596,10 +596,10 @@
         <v>6.091241143731888</v>
       </c>
       <c r="E4" t="n">
-        <v>4.347224991920704</v>
+        <v>4.253268039441625</v>
       </c>
       <c r="F4" t="n">
-        <v>5.315157096071462</v>
+        <v>5.280544611895009</v>
       </c>
     </row>
     <row r="5">
@@ -618,10 +618,10 @@
         <v>3.474342866036952</v>
       </c>
       <c r="E5" t="n">
-        <v>4.307162532296616</v>
+        <v>4.23482579052373</v>
       </c>
       <c r="F5" t="n">
-        <v>5.297408604459279</v>
+        <v>5.381799278591024</v>
       </c>
     </row>
     <row r="6">
@@ -640,10 +640,10 @@
         <v>4.494660689508277</v>
       </c>
       <c r="E6" t="n">
-        <v>4.284532010358539</v>
+        <v>4.250065288889567</v>
       </c>
       <c r="F6" t="n">
-        <v>5.276367645003185</v>
+        <v>5.397817129295025</v>
       </c>
     </row>
     <row r="7">
@@ -662,10 +662,10 @@
         <v>2.419253194704907</v>
       </c>
       <c r="E7" t="n">
-        <v>4.345049114069802</v>
+        <v>4.426556987532945</v>
       </c>
       <c r="F7" t="n">
-        <v>5.2641025390289</v>
+        <v>5.409446822850214</v>
       </c>
     </row>
     <row r="8">
@@ -684,10 +684,10 @@
         <v>3.824239977161246</v>
       </c>
       <c r="E8" t="n">
-        <v>4.094653044167726</v>
+        <v>4.844914623140179</v>
       </c>
       <c r="F8" t="n">
-        <v>5.119213478760006</v>
+        <v>5.215845142480132</v>
       </c>
     </row>
   </sheetData>
@@ -723,7 +723,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.6298132538795471</v>
+        <v>0.6118179559707642</v>
       </c>
     </row>
     <row r="3">
@@ -733,7 +733,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.2954300343990326</v>
+        <v>0.3119166493415833</v>
       </c>
     </row>
     <row r="4">
@@ -743,7 +743,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.04084992036223412</v>
+        <v>0.04496497288346291</v>
       </c>
     </row>
     <row r="5">
@@ -753,27 +753,27 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.01039435900747776</v>
+        <v>0.009291271679103374</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Operational_Risk</t>
+          <t>Credit_Risk</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.008897897787392139</v>
+        <v>0.008198070339858532</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Credit_Risk</t>
+          <t>Operational_Risk</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.007458833511918783</v>
+        <v>0.006927839946001768</v>
       </c>
     </row>
     <row r="8">
@@ -783,7 +783,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.007155647501349449</v>
+        <v>0.006883241701871157</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Final Polish: UI Layouts, Logo Integration, Cache Optimizations, and Chat Architecture Refactor
</commit_message>
<xml_diff>
--- a/reports/risk_summary_report.xlsx
+++ b/reports/risk_summary_report.xlsx
@@ -437,7 +437,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>44702079.31240095</v>
+        <v>44221238.15570626</v>
       </c>
     </row>
     <row r="3">
@@ -447,7 +447,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>44942620.1339686</v>
+        <v>44660169.65620399</v>
       </c>
     </row>
     <row r="4">
@@ -457,7 +457,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2.661852526779229</v>
+        <v>2.703679416981049</v>
       </c>
     </row>
     <row r="5">
@@ -467,7 +467,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>266.1852526779229</v>
+        <v>270.3679416981049</v>
       </c>
     </row>
     <row r="6">
@@ -477,7 +477,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.9988862883439052</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -487,7 +487,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.01372612547129393</v>
+        <v>0.002489626174792647</v>
       </c>
     </row>
   </sheetData>
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -543,19 +543,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1.34068208289301</v>
+        <v>2.493722499534096</v>
       </c>
       <c r="C2" t="n">
-        <v>5.878978490008097</v>
+        <v>5.131987368331983</v>
       </c>
       <c r="D2" t="n">
-        <v>5.47505244242807</v>
+        <v>5.486019274504875</v>
       </c>
       <c r="E2" t="n">
-        <v>4.217095893332942</v>
+        <v>4.363977843344298</v>
       </c>
       <c r="F2" t="n">
-        <v>5.285190094700254</v>
+        <v>5.197377502958843</v>
       </c>
     </row>
     <row r="3">
@@ -565,19 +565,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1.352648849200641</v>
+        <v>3.112547321994142</v>
       </c>
       <c r="C3" t="n">
-        <v>5.791297142984345</v>
+        <v>5.010571645291838</v>
       </c>
       <c r="D3" t="n">
-        <v>3.877120891187244</v>
+        <v>3.867866709237707</v>
       </c>
       <c r="E3" t="n">
-        <v>4.137662937906698</v>
+        <v>4.162656708924589</v>
       </c>
       <c r="F3" t="n">
-        <v>5.421130854100031</v>
+        <v>5.377599154624854</v>
       </c>
     </row>
     <row r="4">
@@ -587,19 +587,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1.476842231040201</v>
+        <v>2.561418946198649</v>
       </c>
       <c r="C4" t="n">
-        <v>5.74641432301136</v>
+        <v>4.990608690987024</v>
       </c>
       <c r="D4" t="n">
-        <v>6.091241143731888</v>
+        <v>6.093823476311049</v>
       </c>
       <c r="E4" t="n">
-        <v>4.156444264019331</v>
+        <v>4.271305530948062</v>
       </c>
       <c r="F4" t="n">
-        <v>5.342730557285626</v>
+        <v>5.429770233952537</v>
       </c>
     </row>
     <row r="5">
@@ -609,19 +609,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1.169459296231764</v>
+        <v>2.528614832523029</v>
       </c>
       <c r="C5" t="n">
-        <v>5.73848753291501</v>
+        <v>4.96080691317336</v>
       </c>
       <c r="D5" t="n">
-        <v>3.474342866036952</v>
+        <v>3.418718099542311</v>
       </c>
       <c r="E5" t="n">
-        <v>4.17164387245862</v>
+        <v>4.180671295851889</v>
       </c>
       <c r="F5" t="n">
-        <v>5.364771642114882</v>
+        <v>5.350290508217662</v>
       </c>
     </row>
     <row r="6">
@@ -631,19 +631,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1.197753654519294</v>
+        <v>2.410909259730387</v>
       </c>
       <c r="C6" t="n">
-        <v>5.825629786265537</v>
+        <v>5.030020251884134</v>
       </c>
       <c r="D6" t="n">
-        <v>4.494660689508277</v>
+        <v>4.508255930946305</v>
       </c>
       <c r="E6" t="n">
-        <v>4.237314661921834</v>
+        <v>4.230629141193819</v>
       </c>
       <c r="F6" t="n">
-        <v>5.309275902572131</v>
+        <v>5.324566637246059</v>
       </c>
     </row>
     <row r="7">
@@ -653,41 +653,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.680321843559095</v>
+        <v>1.484784669857596</v>
       </c>
       <c r="C7" t="n">
-        <v>5.859583401832449</v>
+        <v>5.045717453796541</v>
       </c>
       <c r="D7" t="n">
-        <v>2.419253194704907</v>
+        <v>2.434940969067574</v>
       </c>
       <c r="E7" t="n">
-        <v>4.135198091531637</v>
+        <v>4.271309863257302</v>
       </c>
       <c r="F7" t="n">
-        <v>5.432896655319399</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>UNKNOWN_PRODUCT</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>1.544853976994558</v>
-      </c>
-      <c r="C8" t="n">
-        <v>5.932182131934605</v>
-      </c>
-      <c r="D8" t="n">
-        <v>3.824239977161246</v>
-      </c>
-      <c r="E8" t="n">
-        <v>3.59418831102955</v>
-      </c>
-      <c r="F8" t="n">
-        <v>4.833821398365877</v>
+        <v>5.439025111893626</v>
       </c>
     </row>
   </sheetData>
@@ -723,7 +701,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.6245895624160767</v>
+        <v>0.5790219306945801</v>
       </c>
     </row>
     <row r="3">
@@ -733,7 +711,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.2991340458393097</v>
+        <v>0.3469635844230652</v>
       </c>
     </row>
     <row r="4">
@@ -743,47 +721,47 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.04505334049463272</v>
+        <v>0.04870146512985229</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Operational_Risk</t>
+          <t>Market_Risk</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.009529310278594494</v>
+        <v>0.007192407734692097</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Market_Risk</t>
+          <t>Operational_Risk</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.008225406520068645</v>
+        <v>0.006426296196877956</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Credit_Risk</t>
+          <t>Policy_Tenure_Months</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.008081872016191483</v>
+        <v>0.005854155402630568</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Policy_Tenure_Months</t>
+          <t>Credit_Risk</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.005386462900787592</v>
+        <v>0.00584011897444725</v>
       </c>
     </row>
   </sheetData>

</xml_diff>